<commit_message>
Updated stats matchweek 6
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -33,9 +33,6 @@
     <t>points</t>
   </si>
   <si>
-    <t>a</t>
-  </si>
-  <si>
     <t>b</t>
   </si>
   <si>
@@ -61,6 +58,9 @@
   </si>
   <si>
     <t>j</t>
+  </si>
+  <si>
+    <t>my team</t>
   </si>
 </sst>
 </file>
@@ -414,7 +414,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="B2">
         <v>6</v>
@@ -431,7 +431,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <v>6</v>
@@ -448,7 +448,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>5</v>
@@ -465,7 +465,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>5</v>
@@ -482,7 +482,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -499,7 +499,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>5</v>
@@ -516,7 +516,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>5</v>
@@ -533,7 +533,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>5</v>
@@ -550,7 +550,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>6</v>
@@ -567,7 +567,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>6</v>

</xml_diff>

<commit_message>
Testing new netlify engine
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -33,9 +33,6 @@
     <t>points</t>
   </si>
   <si>
-    <t>b</t>
-  </si>
-  <si>
     <t>c</t>
   </si>
   <si>
@@ -61,6 +58,9 @@
   </si>
   <si>
     <t>my team</t>
+  </si>
+  <si>
+    <t>shit team</t>
   </si>
 </sst>
 </file>
@@ -414,7 +414,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>6</v>
@@ -431,7 +431,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="B3">
         <v>6</v>
@@ -448,7 +448,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4">
         <v>5</v>
@@ -465,7 +465,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5">
         <v>5</v>
@@ -482,7 +482,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -499,7 +499,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>5</v>
@@ -516,7 +516,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>5</v>
@@ -533,7 +533,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9">
         <v>5</v>
@@ -550,7 +550,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10">
         <v>6</v>
@@ -567,7 +567,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11">
         <v>6</v>

</xml_diff>